<commit_message>
Inscriptions : second classeur, mails simplifiés
- le site écrit aussi dans une base secondaire, tenue par un autre
  compte (sheets/base-secondaire.gs) ; une copie ratée n'empêche
  jamais une inscription
- script maître : envoi direct, sans tâche ni file d'attente ; menu
  NTMS pour le mail manuel et les rattrapages
- onglets config auto et config manuel, trouvés quel que soit
  l'orthographe de leur nom
- classeur : menus déroulants sur les colonnes à valeurs fixes
</commit_message>
<xml_diff>
--- a/sheets/ntms-2026-base.xlsx
+++ b/sheets/ntms-2026-base.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="inscriptions" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="config" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="lisez-moi" state="visible" r:id="rId6"/>
+    <sheet sheetId="2" name="config auto" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="config manuel" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="lisez-moi" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="70">
   <si>
     <t>horodatage</t>
   </si>
@@ -82,6 +83,15 @@
   </si>
   <si>
     <t>id_envoi</t>
+  </si>
+  <si>
+    <t>mail_manuel</t>
+  </si>
+  <si>
+    <t>mail_manuel_le</t>
+  </si>
+  <si>
+    <t>erreur_mail_manuel</t>
   </si>
   <si>
     <t>Objet</t>
@@ -142,6 +152,15 @@
     <t>inscriptions</t>
   </si>
   <si>
+    <t>NTMS 2026 — information</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bonjour {{prenom}},
+(Écris ici le message à envoyer à la demande, puis utilise le menu NTMS pour l'envoyer.)
+À très vite,
+AIESEC in Benin</t>
+  </si>
+  <si>
     <t>NTMS 2026 — registre maître des inscriptions</t>
   </si>
   <si>
@@ -163,13 +182,19 @@
     <t xml:space="preserve">  Colonnes tenues par le script : horodatage · reference · mail_envoye · mail_envoye_le · erreur_mail</t>
   </si>
   <si>
+    <t xml:space="preserve">  et, pour le mail manuel : mail_manuel · mail_manuel_le · erreur_mail_manuel</t>
+  </si>
+  <si>
     <t xml:space="preserve">  id_envoi : identifiant technique de chaque envoi, sert à éviter les doublons. Ne pas toucher.</t>
   </si>
   <si>
-    <t>Onglet « config »</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Le contenu du mail envoyé automatiquement à chaque inscrit.</t>
+    <t>Onglet « config auto »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Le contenu du mail envoyé automatiquement à chaque inscrit, au moment de son inscription.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Son contenu se change selon la période : c'est toujours ce mail-là que le site fait partir.</t>
   </si>
   <si>
     <t xml:space="preserve">  Objet et Corps sont obligatoires : sans eux, aucun mail ne part (l'inscription est enregistrée quand même).</t>
@@ -191,6 +216,18 @@
   </si>
   <si>
     <t xml:space="preserve">  Une modification de config prend effet immédiatement, sans redéployer le script.</t>
+  </si>
+  <si>
+    <t>Onglet « config manuel »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Le contenu d'un mail qui ne part JAMAIS tout seul : menu NTMS &gt; Envoyer le mail manuel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Aux lignes sélectionnées, ou à tous ceux qui ne l'ont pas encore reçu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Mêmes champs et mêmes variables que « config auto ».</t>
   </si>
   <si>
     <t>Expéditeur : le compte propriétaire du classeur, celui qui a déployé le script.</t>
@@ -595,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="15" width="14" customWidth="1"/>
@@ -606,9 +643,12 @@
     <col min="21" max="21" width="18" customWidth="1"/>
     <col min="22" max="22" width="15" customWidth="1"/>
     <col min="23" max="23" width="14" customWidth="1"/>
+    <col min="24" max="24" width="15" customWidth="1"/>
+    <col min="25" max="25" width="18" customWidth="1"/>
+    <col min="26" max="26" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -678,8 +718,52 @@
       <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="11">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G2000">
+      <formula1>"Femme,Homme"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="H2:H2000">
+      <formula1>"AIESECer au Bénin,AIESECer d'un autre pays,Pas AIESECer"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I2:I2000">
+      <formula1>"MC,LC"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="J2:J2000">
+      <formula1>"MCP,MCVP,LCP,LCVP,TL,TM"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="K2:K2000">
+      <formula1>"Cotonou,Parakou,Porto-Novo,Abomey-Calavi"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="N2:N2000">
+      <formula1>"Chambre mixte,Chambre non mixte"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="O2:O2000">
+      <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="R2:R2000">
+      <formula1>"oui"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="S2:S2000">
+      <formula1>"oui"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="T2:T2000">
+      <formula1>"oui,non,desactive"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="X2:X2000">
+      <formula1>"oui,non,desactive"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -696,82 +780,82 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" ht="190" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -782,7 +866,94 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="100" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" ht="190" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -790,112 +961,147 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>49</v>
+      <c r="A12" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>50</v>
+      <c r="A13" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Chiffres d'AIESEC in Benin, date du compte à rebours, pièces jointes
- constat : 4 représentations locales et 1000+ jeunes touchés, en plus
  des 20 ans ; trois colonnes sur ordinateur, trois bandes sur téléphone
- compte à rebours : date réglable par NEXT_PUBLIC_DATE_NTMS
- mails : ligne « Pièces jointes » dans les deux onglets de réglage ;
  le fichier est téléchargé par son lien, sans autorisation Drive
- réglages : une adresse collée en lien enrichi est désormais lue
</commit_message>
<xml_diff>
--- a/sheets/ntms-2026-base.xlsx
+++ b/sheets/ntms-2026-base.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="73">
   <si>
     <t>horodatage</t>
   </si>
@@ -146,6 +146,9 @@
     <t>Images</t>
   </si>
   <si>
+    <t>Pièces jointes</t>
+  </si>
+  <si>
     <t>Nom feuille (BD)</t>
   </si>
   <si>
@@ -213,6 +216,12 @@
   </si>
   <si>
     <t xml:space="preserve">  Images : adresses d'images publiques (https://…), séparées par des virgules, affichées en tête du mail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Pièces jointes : liens Google Drive ou adresses https, séparés par des virgules. 25 Mo au total par mail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Un fichier introuvable n'empêche pas le mail de partir : le souci est noté dans la colonne d'erreur.</t>
   </si>
   <si>
     <t xml:space="preserve">  Une modification de config prend effet immédiatement, sans redéployer le script.</t>
@@ -771,6 +780,109 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="100" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" ht="190" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -783,7 +895,7 @@
         <v>26</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -791,7 +903,7 @@
         <v>28</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" ht="190" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -799,7 +911,7 @@
         <v>30</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -807,7 +919,7 @@
         <v>32</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -815,7 +927,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -855,93 +967,6 @@
         <v>42</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="100" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" ht="190" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -953,7 +978,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -961,7 +986,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -971,7 +996,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -981,37 +1006,37 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
@@ -1021,87 +1046,97 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
-        <v>65</v>
+      <c r="A24" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>67</v>
+      <c r="A26" s="5" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>69</v>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>